<commit_message>
Asana task partially done
label names for Shift start and end has been renamed and so is Actual Start Time.
Added the Popup Message for create even and  volunteer.
Data is finally being added on Create event Schedule
Edit is finally editable . Im still working on Multiselect and Calendar.
</commit_message>
<xml_diff>
--- a/Test Upload Excel Files/TestData-Director.xlsx
+++ b/Test Upload Excel Files/TestData-Director.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nyleb\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Semicolon-TomorrowsVoice\Test Upload Excel Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA85A02-06AD-40C0-B36B-759AC8EB43AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9795BB4C-824C-4BD5-86E5-9DCEDEB94425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8310" yWindow="3960" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -462,6 +462,7 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="66.28515625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>